<commit_message>
data: actualización archivos de output v2.3f
</commit_message>
<xml_diff>
--- a/data/output/hallazgos_criticos_auditoria.xlsx
+++ b/data/output/hallazgos_criticos_auditoria.xlsx
@@ -633,7 +633,7 @@
         </is>
       </c>
       <c r="G3" s="4" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>0.3</v>
@@ -668,7 +668,7 @@
         </is>
       </c>
       <c r="G4" s="4" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>0</v>
@@ -699,7 +699,7 @@
         </is>
       </c>
       <c r="G5" s="4" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>0.3</v>
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>0.1</v>
@@ -769,7 +769,7 @@
         </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H7" s="7" t="n">
         <v>0.9</v>
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="G8" s="4" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H8" s="7" t="n">
         <v>0.4</v>
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="G9" s="4" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>19.4</v>
@@ -874,7 +874,7 @@
         </is>
       </c>
       <c r="G10" s="4" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>0.1</v>
@@ -909,7 +909,7 @@
         </is>
       </c>
       <c r="G11" s="4" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>0</v>
@@ -940,7 +940,7 @@
         </is>
       </c>
       <c r="G12" s="4" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H12" s="7" t="n">
         <v>16.3</v>
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="G13" s="4" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H13" s="7" t="n">
         <v>0</v>
@@ -1010,7 +1010,7 @@
         </is>
       </c>
       <c r="G14" s="4" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H14" s="7" t="n">
         <v>0</v>
@@ -1045,7 +1045,7 @@
         </is>
       </c>
       <c r="G15" s="4" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>0</v>
@@ -1080,7 +1080,7 @@
         </is>
       </c>
       <c r="G16" s="4" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H16" s="7" t="n">
         <v>0</v>
@@ -1115,7 +1115,7 @@
         </is>
       </c>
       <c r="G17" s="9" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H17" s="12" t="n">
         <v>20.3</v>
@@ -1150,7 +1150,7 @@
         </is>
       </c>
       <c r="G18" s="4" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H18" s="7" t="n">
         <v>0</v>
@@ -1185,7 +1185,7 @@
         </is>
       </c>
       <c r="G19" s="4" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H19" s="7" t="n">
         <v>0</v>
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="G20" s="4" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H20" s="7" t="n">
         <v>0</v>
@@ -1255,7 +1255,7 @@
         </is>
       </c>
       <c r="G21" s="4" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H21" s="7" t="n">
         <v>0</v>
@@ -1290,7 +1290,7 @@
         </is>
       </c>
       <c r="G22" s="4" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H22" s="7" t="n">
         <v>0.2</v>
@@ -1325,7 +1325,7 @@
         </is>
       </c>
       <c r="G23" s="4" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H23" s="7" t="n">
         <v>0.5</v>
@@ -1360,7 +1360,7 @@
         </is>
       </c>
       <c r="G24" s="4" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H24" s="7" t="n">
         <v>0</v>
@@ -1395,7 +1395,7 @@
         </is>
       </c>
       <c r="G25" s="4" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H25" s="7" t="n">
         <v>5.4</v>
@@ -1430,7 +1430,7 @@
         </is>
       </c>
       <c r="G26" s="4" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H26" s="7" t="n">
         <v>6.8</v>
@@ -1461,7 +1461,7 @@
       </c>
       <c r="F27" s="6" t="inlineStr"/>
       <c r="G27" s="4" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H27" s="7" t="n">
         <v>0</v>
@@ -1492,7 +1492,7 @@
         </is>
       </c>
       <c r="G28" s="4" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H28" s="7" t="n">
         <v>0.1</v>
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="G29" s="4" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H29" s="7" t="n">
         <v>0.2</v>
@@ -1558,7 +1558,7 @@
         </is>
       </c>
       <c r="G30" s="4" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H30" s="7" t="n">
         <v>0.5</v>
@@ -1593,7 +1593,7 @@
         </is>
       </c>
       <c r="G31" s="4" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H31" s="7" t="n">
         <v>0</v>
@@ -1628,7 +1628,7 @@
         </is>
       </c>
       <c r="G32" s="4" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H32" s="7" t="n">
         <v>0.2</v>
@@ -1663,7 +1663,7 @@
         </is>
       </c>
       <c r="G33" s="4" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H33" s="7" t="n">
         <v>17.6</v>
@@ -1694,7 +1694,7 @@
         </is>
       </c>
       <c r="G34" s="4" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H34" s="7" t="n">
         <v>0</v>
@@ -1729,7 +1729,7 @@
         </is>
       </c>
       <c r="G35" s="4" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="H35" s="7" t="n">
         <v>0</v>
@@ -1764,7 +1764,7 @@
         </is>
       </c>
       <c r="G36" s="4" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="H36" s="7" t="n">
         <v>0.1</v>
@@ -1799,7 +1799,7 @@
         </is>
       </c>
       <c r="G37" s="4" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H37" s="7" t="n">
         <v>1</v>
@@ -1834,7 +1834,7 @@
         </is>
       </c>
       <c r="G38" s="4" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H38" s="7" t="n">
         <v>0</v>
@@ -1865,7 +1865,7 @@
         </is>
       </c>
       <c r="G39" s="4" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H39" s="7" t="n">
         <v>0.8</v>
@@ -1900,7 +1900,7 @@
         </is>
       </c>
       <c r="G40" s="4" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H40" s="7" t="n">
         <v>0</v>
@@ -1935,7 +1935,7 @@
         </is>
       </c>
       <c r="G41" s="4" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H41" s="7" t="n">
         <v>0.2</v>
@@ -1970,7 +1970,7 @@
         </is>
       </c>
       <c r="G42" s="9" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H42" s="12" t="n">
         <v>45.7</v>
@@ -2005,7 +2005,7 @@
         </is>
       </c>
       <c r="G43" s="4" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H43" s="7" t="n">
         <v>0.2</v>
@@ -2040,7 +2040,7 @@
         </is>
       </c>
       <c r="G44" s="4" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H44" s="7" t="n">
         <v>0.1</v>
@@ -2075,7 +2075,7 @@
         </is>
       </c>
       <c r="G45" s="4" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H45" s="7" t="n">
         <v>0</v>
@@ -2110,7 +2110,7 @@
         </is>
       </c>
       <c r="G46" s="4" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H46" s="7" t="n">
         <v>0</v>
@@ -2145,7 +2145,7 @@
         </is>
       </c>
       <c r="G47" s="4" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="H47" s="7" t="n">
         <v>0</v>
@@ -2180,7 +2180,7 @@
         </is>
       </c>
       <c r="G48" s="14" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H48" s="17" t="n">
         <v>0</v>
@@ -2215,7 +2215,7 @@
         </is>
       </c>
       <c r="G49" s="14" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="H49" s="17" t="n">
         <v>0</v>
@@ -2250,7 +2250,7 @@
         </is>
       </c>
       <c r="G50" s="14" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="H50" s="17" t="n">
         <v>0</v>
@@ -2285,7 +2285,7 @@
         </is>
       </c>
       <c r="G51" s="14" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H51" s="17" t="n">
         <v>0.6</v>
@@ -2320,7 +2320,7 @@
         </is>
       </c>
       <c r="G52" s="14" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H52" s="17" t="n">
         <v>0.3</v>
@@ -2355,7 +2355,7 @@
         </is>
       </c>
       <c r="G53" s="14" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H53" s="17" t="n">
         <v>0.1</v>
@@ -2390,7 +2390,7 @@
         </is>
       </c>
       <c r="G54" s="14" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H54" s="17" t="n">
         <v>0.5</v>
@@ -2421,7 +2421,7 @@
         </is>
       </c>
       <c r="G55" s="9" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H55" s="12" t="n">
         <v>45.7</v>
@@ -2456,7 +2456,7 @@
         </is>
       </c>
       <c r="G56" s="14" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H56" s="17" t="n">
         <v>5</v>
@@ -2491,7 +2491,7 @@
         </is>
       </c>
       <c r="G57" s="14" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H57" s="17" t="n">
         <v>0.5</v>
@@ -2526,7 +2526,7 @@
         </is>
       </c>
       <c r="G58" s="14" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H58" s="17" t="n">
         <v>0</v>
@@ -2561,7 +2561,7 @@
         </is>
       </c>
       <c r="G59" s="9" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H59" s="12" t="n">
         <v>34.7</v>
@@ -2592,7 +2592,7 @@
         </is>
       </c>
       <c r="G60" s="14" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H60" s="17" t="n">
         <v>0</v>
@@ -2627,7 +2627,7 @@
         </is>
       </c>
       <c r="G61" s="14" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H61" s="17" t="n">
         <v>4.3</v>
@@ -2662,7 +2662,7 @@
         </is>
       </c>
       <c r="G62" s="14" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H62" s="17" t="n">
         <v>11.4</v>
@@ -2697,7 +2697,7 @@
         </is>
       </c>
       <c r="G63" s="14" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H63" s="17" t="n">
         <v>0.3</v>
@@ -2732,7 +2732,7 @@
         </is>
       </c>
       <c r="G64" s="14" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H64" s="17" t="n">
         <v>8.9</v>
@@ -2767,7 +2767,7 @@
         </is>
       </c>
       <c r="G65" s="14" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H65" s="17" t="n">
         <v>0.2</v>
@@ -2802,7 +2802,7 @@
         </is>
       </c>
       <c r="G66" s="14" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H66" s="17" t="n">
         <v>0</v>
@@ -2837,7 +2837,7 @@
         </is>
       </c>
       <c r="G67" s="14" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H67" s="17" t="n">
         <v>0</v>
@@ -2872,7 +2872,7 @@
         </is>
       </c>
       <c r="G68" s="14" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H68" s="17" t="n">
         <v>1.6</v>
@@ -2903,7 +2903,7 @@
         </is>
       </c>
       <c r="G69" s="14" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H69" s="17" t="n">
         <v>3.4</v>
@@ -2938,7 +2938,7 @@
         </is>
       </c>
       <c r="G70" s="14" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H70" s="17" t="n">
         <v>2.3</v>
@@ -2969,7 +2969,7 @@
         </is>
       </c>
       <c r="G71" s="14" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="H71" s="17" t="n">
         <v>0.1</v>
@@ -3000,7 +3000,7 @@
         </is>
       </c>
       <c r="G72" s="14" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H72" s="17" t="n">
         <v>0.4</v>
@@ -3035,7 +3035,7 @@
         </is>
       </c>
       <c r="G73" s="14" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H73" s="17" t="n">
         <v>0</v>
@@ -3070,7 +3070,7 @@
         </is>
       </c>
       <c r="G74" s="14" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H74" s="17" t="n">
         <v>0</v>
@@ -3105,7 +3105,7 @@
         </is>
       </c>
       <c r="G75" s="14" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H75" s="17" t="n">
         <v>0</v>
@@ -3140,7 +3140,7 @@
         </is>
       </c>
       <c r="G76" s="14" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H76" s="17" t="n">
         <v>5.3</v>
@@ -3175,7 +3175,7 @@
         </is>
       </c>
       <c r="G77" s="9" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H77" s="12" t="n">
         <v>42.5</v>
@@ -3210,7 +3210,7 @@
         </is>
       </c>
       <c r="G78" s="14" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H78" s="17" t="n">
         <v>0.1</v>
@@ -3245,7 +3245,7 @@
         </is>
       </c>
       <c r="G79" s="14" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H79" s="17" t="n">
         <v>0</v>
@@ -3280,7 +3280,7 @@
         </is>
       </c>
       <c r="G80" s="14" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H80" s="17" t="n">
         <v>6.3</v>
@@ -3315,7 +3315,7 @@
         </is>
       </c>
       <c r="G81" s="9" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H81" s="12" t="n">
         <v>58.3</v>
@@ -3350,7 +3350,7 @@
         </is>
       </c>
       <c r="G82" s="14" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H82" s="17" t="n">
         <v>0</v>
@@ -3385,7 +3385,7 @@
         </is>
       </c>
       <c r="G83" s="14" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H83" s="17" t="n">
         <v>0</v>
@@ -3420,7 +3420,7 @@
         </is>
       </c>
       <c r="G84" s="14" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H84" s="17" t="n">
         <v>18.7</v>
@@ -3451,7 +3451,7 @@
         </is>
       </c>
       <c r="G85" s="9" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H85" s="12" t="n">
         <v>34.3</v>
@@ -3486,7 +3486,7 @@
         </is>
       </c>
       <c r="G86" s="14" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H86" s="17" t="n">
         <v>0.3</v>
@@ -3517,7 +3517,7 @@
         </is>
       </c>
       <c r="G87" s="14" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H87" s="17" t="n">
         <v>0</v>
@@ -3552,7 +3552,7 @@
         </is>
       </c>
       <c r="G88" s="14" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H88" s="17" t="n">
         <v>0.1</v>
@@ -3587,7 +3587,7 @@
         </is>
       </c>
       <c r="G89" s="14" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H89" s="17" t="n">
         <v>0.1</v>
@@ -3622,7 +3622,7 @@
         </is>
       </c>
       <c r="G90" s="14" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H90" s="17" t="n">
         <v>0</v>
@@ -3653,7 +3653,7 @@
         </is>
       </c>
       <c r="G91" s="14" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H91" s="17" t="n">
         <v>0.1</v>
@@ -3688,7 +3688,7 @@
         </is>
       </c>
       <c r="G92" s="14" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H92" s="17" t="n">
         <v>0.6</v>
@@ -3723,7 +3723,7 @@
         </is>
       </c>
       <c r="G93" s="14" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H93" s="17" t="n">
         <v>11.1</v>
@@ -3758,7 +3758,7 @@
         </is>
       </c>
       <c r="G94" s="14" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H94" s="17" t="n">
         <v>0</v>
@@ -3793,7 +3793,7 @@
         </is>
       </c>
       <c r="G95" s="14" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H95" s="17" t="n">
         <v>0</v>
@@ -3828,7 +3828,7 @@
         </is>
       </c>
       <c r="G96" s="14" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H96" s="17" t="n">
         <v>0.6</v>
@@ -3863,7 +3863,7 @@
         </is>
       </c>
       <c r="G97" s="14" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H97" s="17" t="n">
         <v>0</v>
@@ -3894,7 +3894,7 @@
         </is>
       </c>
       <c r="G98" s="14" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H98" s="17" t="n">
         <v>5.7</v>
@@ -3929,7 +3929,7 @@
         </is>
       </c>
       <c r="G99" s="14" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H99" s="17" t="n">
         <v>0</v>
@@ -3964,7 +3964,7 @@
         </is>
       </c>
       <c r="G100" s="14" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H100" s="17" t="n">
         <v>0.1</v>
@@ -3999,7 +3999,7 @@
         </is>
       </c>
       <c r="G101" s="14" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H101" s="17" t="n">
         <v>0.9</v>
@@ -4034,7 +4034,7 @@
         </is>
       </c>
       <c r="G102" s="14" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H102" s="17" t="n">
         <v>0</v>
@@ -4069,7 +4069,7 @@
         </is>
       </c>
       <c r="G103" s="14" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H103" s="17" t="n">
         <v>0</v>
@@ -4104,7 +4104,7 @@
         </is>
       </c>
       <c r="G104" s="14" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H104" s="17" t="n">
         <v>0</v>
@@ -4139,7 +4139,7 @@
         </is>
       </c>
       <c r="G105" s="14" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H105" s="17" t="n">
         <v>0.2</v>
@@ -4170,7 +4170,7 @@
         </is>
       </c>
       <c r="G106" s="14" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H106" s="17" t="n">
         <v>0.1</v>
@@ -4205,7 +4205,7 @@
         </is>
       </c>
       <c r="G107" s="14" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H107" s="17" t="n">
         <v>0</v>
@@ -4236,7 +4236,7 @@
         </is>
       </c>
       <c r="G108" s="14" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H108" s="17" t="n">
         <v>1.1</v>
@@ -4271,7 +4271,7 @@
         </is>
       </c>
       <c r="G109" s="14" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H109" s="17" t="n">
         <v>0.1</v>
@@ -4306,7 +4306,7 @@
         </is>
       </c>
       <c r="G110" s="14" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H110" s="17" t="n">
         <v>0.6</v>
@@ -4341,7 +4341,7 @@
         </is>
       </c>
       <c r="G111" s="14" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H111" s="17" t="n">
         <v>0</v>
@@ -4376,7 +4376,7 @@
         </is>
       </c>
       <c r="G112" s="14" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H112" s="17" t="n">
         <v>0</v>
@@ -4411,7 +4411,7 @@
         </is>
       </c>
       <c r="G113" s="14" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H113" s="17" t="n">
         <v>0</v>
@@ -4446,7 +4446,7 @@
         </is>
       </c>
       <c r="G114" s="14" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H114" s="17" t="n">
         <v>0.1</v>
@@ -4481,7 +4481,7 @@
         </is>
       </c>
       <c r="G115" s="14" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H115" s="17" t="n">
         <v>0</v>
@@ -4516,7 +4516,7 @@
         </is>
       </c>
       <c r="G116" s="14" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H116" s="17" t="n">
         <v>0</v>
@@ -4551,7 +4551,7 @@
         </is>
       </c>
       <c r="G117" s="9" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H117" s="12" t="n">
         <v>32</v>
@@ -4586,7 +4586,7 @@
         </is>
       </c>
       <c r="G118" s="14" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H118" s="17" t="n">
         <v>0.1</v>
@@ -4621,7 +4621,7 @@
         </is>
       </c>
       <c r="G119" s="14" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H119" s="17" t="n">
         <v>0.6</v>
@@ -4656,7 +4656,7 @@
         </is>
       </c>
       <c r="G120" s="14" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H120" s="17" t="n">
         <v>0</v>
@@ -4691,7 +4691,7 @@
         </is>
       </c>
       <c r="G121" s="14" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H121" s="17" t="n">
         <v>0</v>
@@ -4722,7 +4722,7 @@
         </is>
       </c>
       <c r="G122" s="14" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H122" s="17" t="n">
         <v>0</v>
@@ -4757,7 +4757,7 @@
         </is>
       </c>
       <c r="G123" s="14" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H123" s="17" t="n">
         <v>0</v>
@@ -4792,7 +4792,7 @@
         </is>
       </c>
       <c r="G124" s="14" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H124" s="17" t="n">
         <v>0</v>
@@ -4827,7 +4827,7 @@
         </is>
       </c>
       <c r="G125" s="14" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H125" s="17" t="n">
         <v>0</v>
@@ -4862,7 +4862,7 @@
         </is>
       </c>
       <c r="G126" s="14" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H126" s="17" t="n">
         <v>0.2</v>
@@ -4897,7 +4897,7 @@
         </is>
       </c>
       <c r="G127" s="14" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H127" s="17" t="n">
         <v>0.1</v>
@@ -4932,7 +4932,7 @@
         </is>
       </c>
       <c r="G128" s="14" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H128" s="17" t="n">
         <v>11.3</v>
@@ -4967,7 +4967,7 @@
         </is>
       </c>
       <c r="G129" s="9" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H129" s="12" t="n">
         <v>26.4</v>
@@ -5002,7 +5002,7 @@
         </is>
       </c>
       <c r="G130" s="14" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H130" s="17" t="n">
         <v>0</v>
@@ -5037,7 +5037,7 @@
         </is>
       </c>
       <c r="G131" s="14" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H131" s="17" t="n">
         <v>0.6</v>
@@ -5072,7 +5072,7 @@
         </is>
       </c>
       <c r="G132" s="14" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H132" s="17" t="n">
         <v>0.2</v>
@@ -5107,7 +5107,7 @@
         </is>
       </c>
       <c r="G133" s="14" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H133" s="17" t="n">
         <v>4.4</v>
@@ -5142,7 +5142,7 @@
         </is>
       </c>
       <c r="G134" s="14" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H134" s="17" t="n">
         <v>0</v>
@@ -5173,7 +5173,7 @@
         </is>
       </c>
       <c r="G135" s="14" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H135" s="17" t="n">
         <v>0.8</v>
@@ -5208,7 +5208,7 @@
         </is>
       </c>
       <c r="G136" s="14" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H136" s="17" t="n">
         <v>17.4</v>
@@ -5243,7 +5243,7 @@
         </is>
       </c>
       <c r="G137" s="14" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H137" s="17" t="n">
         <v>0</v>
@@ -5274,7 +5274,7 @@
       </c>
       <c r="F138" s="11" t="inlineStr"/>
       <c r="G138" s="9" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H138" s="12" t="n">
         <v>44.6</v>
@@ -5309,7 +5309,7 @@
         </is>
       </c>
       <c r="G139" s="14" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H139" s="17" t="n">
         <v>0</v>
@@ -5344,7 +5344,7 @@
         </is>
       </c>
       <c r="G140" s="14" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H140" s="17" t="n">
         <v>0</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="G141" s="14" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H141" s="17" t="n">
         <v>0.1</v>
@@ -5414,7 +5414,7 @@
         </is>
       </c>
       <c r="G142" s="14" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H142" s="17" t="n">
         <v>0</v>
@@ -5449,7 +5449,7 @@
         </is>
       </c>
       <c r="G143" s="14" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H143" s="17" t="n">
         <v>0</v>
@@ -5484,7 +5484,7 @@
         </is>
       </c>
       <c r="G144" s="14" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H144" s="17" t="n">
         <v>0.4</v>
@@ -5515,7 +5515,7 @@
         </is>
       </c>
       <c r="G145" s="14" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H145" s="17" t="n">
         <v>0</v>
@@ -5550,7 +5550,7 @@
         </is>
       </c>
       <c r="G146" s="9" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H146" s="12" t="n">
         <v>54.2</v>
@@ -5585,7 +5585,7 @@
         </is>
       </c>
       <c r="G147" s="14" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H147" s="17" t="n">
         <v>3.4</v>
@@ -5620,7 +5620,7 @@
         </is>
       </c>
       <c r="G148" s="14" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H148" s="17" t="n">
         <v>0.2</v>
@@ -5655,7 +5655,7 @@
         </is>
       </c>
       <c r="G149" s="14" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H149" s="17" t="n">
         <v>0</v>
@@ -5690,7 +5690,7 @@
         </is>
       </c>
       <c r="G150" s="14" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H150" s="17" t="n">
         <v>0</v>
@@ -5725,7 +5725,7 @@
         </is>
       </c>
       <c r="G151" s="14" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H151" s="17" t="n">
         <v>0</v>
@@ -5760,7 +5760,7 @@
         </is>
       </c>
       <c r="G152" s="14" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H152" s="17" t="n">
         <v>5.4</v>
@@ -5795,7 +5795,7 @@
         </is>
       </c>
       <c r="G153" s="14" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H153" s="17" t="n">
         <v>0</v>
@@ -5830,7 +5830,7 @@
         </is>
       </c>
       <c r="G154" s="14" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H154" s="17" t="n">
         <v>0</v>
@@ -5865,7 +5865,7 @@
         </is>
       </c>
       <c r="G155" s="14" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H155" s="17" t="n">
         <v>0.2</v>
@@ -5900,7 +5900,7 @@
         </is>
       </c>
       <c r="G156" s="14" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H156" s="17" t="n">
         <v>0</v>
@@ -5931,7 +5931,7 @@
         </is>
       </c>
       <c r="G157" s="14" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H157" s="17" t="n">
         <v>0.7</v>
@@ -5966,7 +5966,7 @@
         </is>
       </c>
       <c r="G158" s="14" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H158" s="17" t="n">
         <v>8.300000000000001</v>
@@ -6001,7 +6001,7 @@
         </is>
       </c>
       <c r="G159" s="14" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H159" s="17" t="n">
         <v>0</v>
@@ -6036,7 +6036,7 @@
         </is>
       </c>
       <c r="G160" s="14" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H160" s="17" t="n">
         <v>0.2</v>
@@ -6071,7 +6071,7 @@
         </is>
       </c>
       <c r="G161" s="14" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H161" s="17" t="n">
         <v>0</v>
@@ -6106,7 +6106,7 @@
         </is>
       </c>
       <c r="G162" s="14" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H162" s="17" t="n">
         <v>0</v>
@@ -6141,7 +6141,7 @@
         </is>
       </c>
       <c r="G163" s="14" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H163" s="17" t="n">
         <v>0</v>
@@ -6172,7 +6172,7 @@
         </is>
       </c>
       <c r="G164" s="14" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H164" s="17" t="n">
         <v>0</v>
@@ -6207,7 +6207,7 @@
         </is>
       </c>
       <c r="G165" s="14" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H165" s="17" t="n">
         <v>0.1</v>
@@ -6238,7 +6238,7 @@
         </is>
       </c>
       <c r="G166" s="14" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H166" s="17" t="n">
         <v>0.1</v>
@@ -6273,7 +6273,7 @@
         </is>
       </c>
       <c r="G167" s="14" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H167" s="17" t="n">
         <v>0</v>
@@ -6308,7 +6308,7 @@
         </is>
       </c>
       <c r="G168" s="14" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H168" s="17" t="n">
         <v>0.3</v>
@@ -6343,7 +6343,7 @@
         </is>
       </c>
       <c r="G169" s="14" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H169" s="17" t="n">
         <v>0</v>
@@ -6378,7 +6378,7 @@
         </is>
       </c>
       <c r="G170" s="14" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H170" s="17" t="n">
         <v>0.3</v>
@@ -6413,7 +6413,7 @@
         </is>
       </c>
       <c r="G171" s="14" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H171" s="17" t="n">
         <v>0</v>
@@ -6448,7 +6448,7 @@
         </is>
       </c>
       <c r="G172" s="14" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H172" s="17" t="n">
         <v>7.5</v>
@@ -6483,7 +6483,7 @@
         </is>
       </c>
       <c r="G173" s="14" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H173" s="17" t="n">
         <v>9.300000000000001</v>
@@ -6518,7 +6518,7 @@
         </is>
       </c>
       <c r="G174" s="9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H174" s="12" t="n">
         <v>50.8</v>
@@ -6553,7 +6553,7 @@
         </is>
       </c>
       <c r="G175" s="14" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H175" s="17" t="n">
         <v>2.8</v>
@@ -6588,7 +6588,7 @@
         </is>
       </c>
       <c r="G176" s="14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H176" s="17" t="n">
         <v>0</v>
@@ -6623,7 +6623,7 @@
         </is>
       </c>
       <c r="G177" s="14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H177" s="17" t="n">
         <v>0</v>
@@ -6658,7 +6658,7 @@
         </is>
       </c>
       <c r="G178" s="14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H178" s="17" t="n">
         <v>0</v>
@@ -6693,7 +6693,7 @@
         </is>
       </c>
       <c r="G179" s="14" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H179" s="17" t="n">
         <v>0.2</v>
@@ -6728,7 +6728,7 @@
         </is>
       </c>
       <c r="G180" s="14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H180" s="17" t="n">
         <v>0</v>
@@ -6763,7 +6763,7 @@
         </is>
       </c>
       <c r="G181" s="14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H181" s="17" t="n">
         <v>0</v>
@@ -6798,7 +6798,7 @@
         </is>
       </c>
       <c r="G182" s="14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H182" s="17" t="n">
         <v>0.3</v>
@@ -6833,7 +6833,7 @@
         </is>
       </c>
       <c r="G183" s="14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H183" s="17" t="n">
         <v>0.1</v>
@@ -6868,7 +6868,7 @@
         </is>
       </c>
       <c r="G184" s="14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H184" s="17" t="n">
         <v>0</v>
@@ -6903,7 +6903,7 @@
         </is>
       </c>
       <c r="G185" s="14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H185" s="17" t="n">
         <v>0</v>
@@ -6938,7 +6938,7 @@
         </is>
       </c>
       <c r="G186" s="14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H186" s="17" t="n">
         <v>0.1</v>

</xml_diff>